<commit_message>
feat: 달력 from~to 설정, excel 기능 고도화
</commit_message>
<xml_diff>
--- a/templates/단위테스트 템플릿.xlsx
+++ b/templates/단위테스트 템플릿.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KB099\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\promptcase-studio\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{417DCB22-615E-431B-9915-6130C5960FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA1D7FB7-36D1-480E-88BE-4E1321105F63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12" yWindow="12" windowWidth="23016" windowHeight="12216" xr2:uid="{AD02B665-237F-4D57-887F-DAAC4116AF57}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AD02B665-237F-4D57-887F-DAAC4116AF57}"/>
   </bookViews>
   <sheets>
     <sheet name="프로그램 정보" sheetId="3" r:id="rId1"/>
@@ -349,7 +349,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -377,38 +377,35 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -758,44 +755,44 @@
   <sheetData>
     <row r="1" spans="2:7" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="9"/>
-    </row>
-    <row r="3" spans="2:7" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="10" t="s">
+      <c r="C2" s="18"/>
+    </row>
+    <row r="3" spans="2:7" s="10" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="2:7" s="15" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="12" t="s">
+    <row r="4" spans="2:7" s="14" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="16" t="s">
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="14"/>
+      <c r="G4" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -903,19 +900,19 @@
       </c>
     </row>
     <row r="3" spans="2:3" ht="100.05" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="15" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="4"/>
     </row>
     <row r="4" spans="2:3" ht="100.05" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="16" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="6"/>
     </row>
     <row r="5" spans="2:3" ht="199.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="17" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="8"/>

</xml_diff>